<commit_message>
feat: add email reservation API with nodemailer integration
- Implemented a new API route for handling reservation emails using nodemailer.
- Added HTML email template for reservation details.
- Updated package.json and pnpm-lock.yaml to include nodemailer and its types.
- Removed globals.css as part of styling refactor.
- Added various media files for tours and transfers.
</commit_message>
<xml_diff>
--- a/public/media/transport ashab tours.xlsx
+++ b/public/media/transport ashab tours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ashab-tours\ashba-tour\public\media\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07869B83-0FA7-4E09-B022-1D903C39BDAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E7D032-BD8D-4CEC-8039-FB12852CC3C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-100" yWindow="-100" windowWidth="26836" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -249,13 +249,7 @@
  Stability: Well-maintained suspension systems for winding mountain roads.</t>
   </si>
   <si>
-    <t xml:space="preserve">ExcursionTerreD'amanar </t>
-  </si>
-  <si>
     <t>Terresd'Amanar Adventure</t>
-  </si>
-  <si>
-    <t>ExcursionTerreD'amanar.png</t>
   </si>
   <si>
     <t>ExcursionOurikaOuirganImlilOukaimden</t>
@@ -603,6 +597,12 @@
   </si>
   <si>
     <t>ForfairtCircuit.png</t>
+  </si>
+  <si>
+    <t>ExcursionTerreD_amanar.png</t>
+  </si>
+  <si>
+    <t>ExcursionTerreD_amanar</t>
   </si>
 </sst>
 </file>
@@ -1365,10 +1365,10 @@
     </row>
     <row r="17" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>39</v>
@@ -1380,7 +1380,7 @@
         <v>14</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>72</v>
+        <v>184</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>63</v>
@@ -1394,13 +1394,13 @@
     </row>
     <row r="18" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>13</v>
@@ -1409,7 +1409,7 @@
         <v>14</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>69</v>
@@ -1423,10 +1423,10 @@
     </row>
     <row r="19" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>39</v>
@@ -1438,7 +1438,7 @@
         <v>14</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>69</v>
@@ -1452,10 +1452,10 @@
     </row>
     <row r="20" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>39</v>
@@ -1467,7 +1467,7 @@
         <v>14</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>69</v>
@@ -1481,10 +1481,10 @@
     </row>
     <row r="21" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>39</v>
@@ -1496,10 +1496,10 @@
         <v>14</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>64</v>
@@ -1510,10 +1510,10 @@
     </row>
     <row r="22" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>39</v>
@@ -1525,10 +1525,10 @@
         <v>14</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>64</v>
@@ -1539,10 +1539,10 @@
     </row>
     <row r="23" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>39</v>
@@ -1554,10 +1554,10 @@
         <v>14</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>64</v>
@@ -1568,10 +1568,10 @@
     </row>
     <row r="24" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>39</v>
@@ -1583,10 +1583,10 @@
         <v>14</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>64</v>
@@ -1597,10 +1597,10 @@
     </row>
     <row r="25" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>39</v>
@@ -1612,10 +1612,10 @@
         <v>14</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>64</v>
@@ -1626,10 +1626,10 @@
     </row>
     <row r="26" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>39</v>
@@ -1641,10 +1641,10 @@
         <v>14</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>64</v>
@@ -1655,10 +1655,10 @@
     </row>
     <row r="27" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>39</v>
@@ -1670,10 +1670,10 @@
         <v>14</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>64</v>
@@ -1684,10 +1684,10 @@
     </row>
     <row r="28" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>39</v>
@@ -1699,10 +1699,10 @@
         <v>14</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>64</v>
@@ -1713,10 +1713,10 @@
     </row>
     <row r="29" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>39</v>
@@ -1728,10 +1728,10 @@
         <v>14</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>64</v>
@@ -1742,10 +1742,10 @@
     </row>
     <row r="30" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>39</v>
@@ -1757,13 +1757,13 @@
         <v>14</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J30" s="2" t="b">
         <v>0</v>
@@ -1771,10 +1771,10 @@
     </row>
     <row r="31" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>39</v>
@@ -1786,13 +1786,13 @@
         <v>14</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J31" s="2" t="b">
         <v>0</v>
@@ -1800,10 +1800,10 @@
     </row>
     <row r="32" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>39</v>
@@ -1815,13 +1815,13 @@
         <v>14</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J32" s="2" t="b">
         <v>0</v>
@@ -1829,10 +1829,10 @@
     </row>
     <row r="33" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>39</v>
@@ -1844,13 +1844,13 @@
         <v>14</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J33" s="2" t="b">
         <v>0</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="34" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>12</v>
@@ -1873,13 +1873,13 @@
         <v>14</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J34" s="2" t="b">
         <v>0</v>
@@ -1887,10 +1887,10 @@
     </row>
     <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>39</v>
@@ -1902,13 +1902,13 @@
         <v>14</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J35" s="2" t="b">
         <v>0</v>
@@ -1916,10 +1916,10 @@
     </row>
     <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>39</v>
@@ -1931,13 +1931,13 @@
         <v>14</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J36" s="2" t="b">
         <v>0</v>
@@ -1945,10 +1945,10 @@
     </row>
     <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>39</v>
@@ -1960,13 +1960,13 @@
         <v>14</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J37" s="2" t="b">
         <v>0</v>
@@ -1974,10 +1974,10 @@
     </row>
     <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>39</v>
@@ -1989,13 +1989,13 @@
         <v>14</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J38" s="2" t="b">
         <v>0</v>
@@ -2003,10 +2003,10 @@
     </row>
     <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>39</v>
@@ -2018,13 +2018,13 @@
         <v>14</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J39" s="2" t="b">
         <v>0</v>
@@ -2032,10 +2032,10 @@
     </row>
     <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>39</v>
@@ -2047,13 +2047,13 @@
         <v>14</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J40" s="2" t="b">
         <v>0</v>
@@ -2061,10 +2061,10 @@
     </row>
     <row r="41" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>39</v>
@@ -2076,13 +2076,13 @@
         <v>14</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J41" s="2" t="b">
         <v>0</v>
@@ -2090,10 +2090,10 @@
     </row>
     <row r="42" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>39</v>
@@ -2105,13 +2105,13 @@
         <v>14</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J42" s="2" t="b">
         <v>0</v>
@@ -2119,10 +2119,10 @@
     </row>
     <row r="43" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A43" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>39</v>
@@ -2134,13 +2134,13 @@
         <v>14</v>
       </c>
       <c r="G43" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="I43" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="H43" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="J43" s="2" t="b">
         <v>0</v>
@@ -2148,10 +2148,10 @@
     </row>
     <row r="44" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>39</v>
@@ -2163,13 +2163,13 @@
         <v>14</v>
       </c>
       <c r="G44" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="I44" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="H44" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="J44" s="2" t="b">
         <v>0</v>
@@ -2177,10 +2177,10 @@
     </row>
     <row r="45" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>39</v>
@@ -2192,13 +2192,13 @@
         <v>14</v>
       </c>
       <c r="G45" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="I45" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="H45" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="J45" s="2" t="b">
         <v>0</v>
@@ -2206,10 +2206,10 @@
     </row>
     <row r="46" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A46" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>39</v>
@@ -2221,13 +2221,13 @@
         <v>14</v>
       </c>
       <c r="G46" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="I46" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="H46" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="J46" s="2" t="b">
         <v>0</v>
@@ -2235,10 +2235,10 @@
     </row>
     <row r="47" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A47" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>39</v>
@@ -2250,13 +2250,13 @@
         <v>14</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J47" s="2" t="b">
         <v>0</v>
@@ -2264,10 +2264,10 @@
     </row>
     <row r="48" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A48" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>39</v>
@@ -2279,13 +2279,13 @@
         <v>14</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J48" s="2" t="b">
         <v>0</v>
@@ -2293,10 +2293,10 @@
     </row>
     <row r="49" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A49" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>39</v>
@@ -2308,13 +2308,13 @@
         <v>14</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J49" s="2" t="b">
         <v>0</v>
@@ -2322,10 +2322,10 @@
     </row>
     <row r="50" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A50" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>39</v>
@@ -2337,13 +2337,13 @@
         <v>14</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J50" s="2" t="b">
         <v>0</v>
@@ -2351,10 +2351,10 @@
     </row>
     <row r="51" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A51" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>39</v>
@@ -2366,13 +2366,13 @@
         <v>14</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J51" s="2" t="b">
         <v>0</v>
@@ -2380,10 +2380,10 @@
     </row>
     <row r="52" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>39</v>
@@ -2395,13 +2395,13 @@
         <v>14</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J52" s="2" t="b">
         <v>0</v>

</xml_diff>